<commit_message>
feat: adicionado relatorio leitura que utiliza o arquivo de modelo corretamente
</commit_message>
<xml_diff>
--- a/SINOSBYTE-TEMPLATE-Vazio.xlsx
+++ b/SINOSBYTE-TEMPLATE-Vazio.xlsx
@@ -29,12 +29,33 @@
     <t>Mês:</t>
   </si>
   <si>
+    <t>Preencha apenas as células amarelas (Entrada, Saída Almoço, Retorno Almoço, Saída). O Total de Horas e o Total do Mês são calculados automaticamente. O mês/ano é definido na aba Consolidado.</t>
+  </si>
+  <si>
+    <t>Colaborador:</t>
+  </si>
+  <si>
+    <t>Cargo:</t>
+  </si>
+  <si>
+    <t>Empresa:</t>
+  </si>
+  <si>
+    <t>Squad:</t>
+  </si>
+  <si>
+    <t>Valor Hora (R$):</t>
+  </si>
+  <si>
     <t>Revise a coluna VALOR HORA (em azul) se houve reajuste. As colunas TOTAL DE HORAS e TOTAL R$ MENSAL são calculadas automaticamente a partir da aba de cada colaborador.</t>
   </si>
   <si>
     <t>COLABORADOR</t>
   </si>
   <si>
+    <t>Mês/Ano:</t>
+  </si>
+  <si>
     <t>CARGO/FUNÇÃO</t>
   </si>
   <si>
@@ -65,52 +86,31 @@
     <t>MÊS</t>
   </si>
   <si>
-    <t>Preencha apenas as células amarelas (Entrada, Saída Almoço, Retorno Almoço, Saída). O Total de Horas e o Total do Mês são calculados automaticamente. O mês/ano é definido na aba Consolidado.</t>
-  </si>
-  <si>
-    <t>Colaborador:</t>
-  </si>
-  <si>
-    <t>Cargo:</t>
-  </si>
-  <si>
-    <t>Empresa:</t>
-  </si>
-  <si>
-    <t>Squad:</t>
-  </si>
-  <si>
-    <t>Valor Hora (R$):</t>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Dia da Semana</t>
+  </si>
+  <si>
+    <t>Entrada</t>
+  </si>
+  <si>
+    <t>Saída Almoço</t>
+  </si>
+  <si>
+    <t>Retorno Almoço</t>
+  </si>
+  <si>
+    <t>Saída</t>
+  </si>
+  <si>
+    <t>Total Horas</t>
+  </si>
+  <si>
+    <t>Observações</t>
   </si>
   <si>
     <t>TOTAL GERAL</t>
-  </si>
-  <si>
-    <t>Mês/Ano:</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Dia da Semana</t>
-  </si>
-  <si>
-    <t>Entrada</t>
-  </si>
-  <si>
-    <t>Saída Almoço</t>
-  </si>
-  <si>
-    <t>Retorno Almoço</t>
-  </si>
-  <si>
-    <t>Saída</t>
-  </si>
-  <si>
-    <t>Total Horas</t>
-  </si>
-  <si>
-    <t>Observações</t>
   </si>
   <si>
     <t>TOTAL HORAS DO MÊS</t>
@@ -195,14 +195,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -243,33 +243,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="9" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="2" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="14" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="2" fillId="4" fontId="3" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="5" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="14" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="5" fontId="5" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf borderId="2" fillId="5" fontId="3" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="2" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="2" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
@@ -515,7 +515,6 @@
     <col customWidth="1" min="9" max="9" width="14.0"/>
     <col customWidth="1" min="10" max="10" width="16.0"/>
     <col customWidth="1" min="11" max="11" width="12.0"/>
-    <col customWidth="1" min="12" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,81 +539,102 @@
       <c r="G4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="5" t="str">
+        <f>CHOOSE(B4,"JANEIRO","FEVEREIRO","MARÇO","ABRIL","MAIO","JUNHO","JULHO","AGOSTO","SETEMBRO","OUTUBRO","NOVEMBRO","DEZEMBRO")</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>16</v>
       </c>
+      <c r="E8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="7"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="12">
+        <f>'Nome Colaborador'!G40</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="13">
+        <f t="shared" ref="J9:J10" si="1">H9*I9</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="str">
+        <f t="shared" ref="K9:K10" si="2">$H$4</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="7"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="12" t="str">
+        <f>'Ringo Star'!G40</f>
+        <v>#REF!</v>
+      </c>
+      <c r="J10" s="13" t="str">
+        <f t="shared" si="1"/>
+        <v>#REF!</v>
+      </c>
+      <c r="K10" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="11">
-      <c r="H11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11" s="14">
+      <c r="H11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="J11" s="17" t="str">
         <f>SUM(J9:J10)</f>
-        <v>0</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1623,668 +1643,667 @@
     <col customWidth="1" min="4" max="5" width="14.0"/>
     <col customWidth="1" min="6" max="7" width="12.0"/>
     <col customWidth="1" min="8" max="8" width="24.0"/>
-    <col customWidth="1" min="9" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
-        <f>"REGISTRO DE PONTO — NOME — SINOSBYTE — " &amp; Consolidado!$H$4 &amp; "/" &amp; Consolidado!$E$4</f>
-        <v>REGISTRO DE PONTO — NOME — SINOSBYTE — /</v>
+        <f>"REGISTRO DE PONTO — George Harrison — SINOSBYTE — " &amp; Consolidado!$H$4 &amp; "/" &amp; Consolidado!$E$4</f>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B4" s="5"/>
       <c r="D4" s="3" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E4" s="5"/>
       <c r="G4" s="3" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="H4" s="5"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B5" s="5"/>
       <c r="D5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="13" t="str">
+        <v>10</v>
+      </c>
+      <c r="E5" s="6" t="str">
         <f>Consolidado!H9</f>
         <v/>
       </c>
       <c r="G5" s="3" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="H5" s="5" t="str">
         <f>Consolidado!$H$4&amp;"/"&amp;Consolidado!$E$4</f>
-        <v>/</v>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="C7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E7" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="F7" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="G7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="H7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="15" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="str">
+      <c r="A8" s="14" t="str">
         <f>IF(1&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,1),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B8" s="7" t="str">
+      <c r="B8" s="8" t="str">
         <f t="shared" ref="B8:B38" si="1">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
       <c r="G8" s="18" t="str">
         <f t="shared" ref="G8:G38" si="2">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
         <v/>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="str">
+      <c r="A9" s="14" t="str">
         <f>IF(2&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,2),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B9" s="7" t="str">
+      <c r="B9" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
       <c r="G9" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="8"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="str">
+      <c r="A10" s="14" t="str">
         <f>IF(3&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,3),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B10" s="7" t="str">
+      <c r="B10" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
       <c r="G10" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="8"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="str">
+      <c r="A11" s="14" t="str">
         <f>IF(4&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,4),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B11" s="7" t="str">
+      <c r="B11" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
       <c r="G11" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="8"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="str">
+      <c r="A12" s="14" t="str">
         <f>IF(5&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,5),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B12" s="7" t="str">
+      <c r="B12" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
       <c r="G12" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="8"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="str">
+      <c r="A13" s="14" t="str">
         <f>IF(6&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,6),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B13" s="7" t="str">
+      <c r="B13" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
       <c r="G13" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="8"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="str">
+      <c r="A14" s="14" t="str">
         <f>IF(7&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,7),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B14" s="7" t="str">
+      <c r="B14" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
       <c r="G14" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="8"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="str">
+      <c r="A15" s="14" t="str">
         <f>IF(8&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,8),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B15" s="7" t="str">
+      <c r="B15" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
       <c r="G15" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="8"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="str">
+      <c r="A16" s="14" t="str">
         <f>IF(9&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,9),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B16" s="7" t="str">
+      <c r="B16" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
       <c r="G16" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="8"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="str">
+      <c r="A17" s="14" t="str">
         <f>IF(10&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,10),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B17" s="7" t="str">
+      <c r="B17" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
       <c r="G17" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="8"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="str">
+      <c r="A18" s="14" t="str">
         <f>IF(11&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,11),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B18" s="7" t="str">
+      <c r="B18" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
       <c r="G18" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H18" s="7"/>
+      <c r="H18" s="8"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="str">
+      <c r="A19" s="14" t="str">
         <f>IF(12&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,12),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B19" s="7" t="str">
+      <c r="B19" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
       <c r="G19" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="8"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="str">
+      <c r="A20" s="14" t="str">
         <f>IF(13&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,13),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B20" s="7" t="str">
+      <c r="B20" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
       <c r="G20" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="8"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="16" t="str">
+      <c r="A21" s="14" t="str">
         <f>IF(14&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,14),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B21" s="7" t="str">
+      <c r="B21" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
       <c r="G21" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="8"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="16" t="str">
+      <c r="A22" s="14" t="str">
         <f>IF(15&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,15),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B22" s="7" t="str">
+      <c r="B22" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
       <c r="G22" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="8"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="16" t="str">
+      <c r="A23" s="14" t="str">
         <f>IF(16&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,16),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B23" s="7" t="str">
+      <c r="B23" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
       <c r="G23" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H23" s="7"/>
+      <c r="H23" s="8"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="16" t="str">
+      <c r="A24" s="14" t="str">
         <f>IF(17&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,17),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B24" s="7" t="str">
+      <c r="B24" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
       <c r="G24" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H24" s="7"/>
+      <c r="H24" s="8"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="16" t="str">
+      <c r="A25" s="14" t="str">
         <f>IF(18&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,18),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B25" s="7" t="str">
+      <c r="B25" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
       <c r="G25" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H25" s="7"/>
+      <c r="H25" s="8"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="16" t="str">
+      <c r="A26" s="14" t="str">
         <f>IF(19&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,19),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B26" s="7" t="str">
+      <c r="B26" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
       <c r="G26" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H26" s="7"/>
+      <c r="H26" s="8"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="16" t="str">
+      <c r="A27" s="14" t="str">
         <f>IF(20&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,20),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B27" s="7" t="str">
+      <c r="B27" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
       <c r="G27" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H27" s="7"/>
+      <c r="H27" s="8"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="16" t="str">
+      <c r="A28" s="14" t="str">
         <f>IF(21&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,21),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B28" s="7" t="str">
+      <c r="B28" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
       <c r="G28" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H28" s="7"/>
+      <c r="H28" s="8"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="16" t="str">
+      <c r="A29" s="14" t="str">
         <f>IF(22&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,22),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B29" s="7" t="str">
+      <c r="B29" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
       <c r="G29" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H29" s="7"/>
+      <c r="H29" s="8"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="16" t="str">
+      <c r="A30" s="14" t="str">
         <f>IF(23&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,23),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B30" s="7" t="str">
+      <c r="B30" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
       <c r="G30" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H30" s="7"/>
+      <c r="H30" s="8"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="16" t="str">
+      <c r="A31" s="14" t="str">
         <f>IF(24&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,24),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B31" s="7" t="str">
+      <c r="B31" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
       <c r="G31" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H31" s="7"/>
+      <c r="H31" s="8"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="16" t="str">
+      <c r="A32" s="14" t="str">
         <f>IF(25&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,25),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B32" s="7" t="str">
+      <c r="B32" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
       <c r="G32" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H32" s="7"/>
+      <c r="H32" s="8"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="16" t="str">
+      <c r="A33" s="14" t="str">
         <f>IF(26&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,26),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B33" s="7" t="str">
+      <c r="B33" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
       <c r="G33" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H33" s="7"/>
+      <c r="H33" s="8"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="16" t="str">
+      <c r="A34" s="14" t="str">
         <f>IF(27&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,27),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B34" s="7" t="str">
+      <c r="B34" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
       <c r="G34" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H34" s="7"/>
+      <c r="H34" s="8"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="16" t="str">
+      <c r="A35" s="14" t="str">
         <f>IF(28&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,28),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B35" s="7" t="str">
+      <c r="B35" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
       <c r="G35" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H35" s="7"/>
+      <c r="H35" s="8"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="16" t="str">
+      <c r="A36" s="14" t="str">
         <f>IF(29&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,29),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B36" s="7" t="str">
+      <c r="B36" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
       <c r="G36" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H36" s="7"/>
+      <c r="H36" s="8"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="16" t="str">
+      <c r="A37" s="14" t="str">
         <f>IF(30&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,30),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B37" s="7" t="str">
+      <c r="B37" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
       <c r="G37" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H37" s="7"/>
+      <c r="H37" s="8"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="16" t="str">
+      <c r="A38" s="14" t="str">
         <f>IF(31&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,31),"")</f>
         <v>#NUM!</v>
       </c>
-      <c r="B38" s="7" t="str">
+      <c r="B38" s="8" t="str">
         <f t="shared" si="1"/>
         <v>#NUM!</v>
       </c>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
       <c r="G38" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="H38" s="7"/>
+      <c r="H38" s="8"/>
     </row>
     <row r="39" ht="15.75" customHeight="1"/>
     <row r="40" ht="15.75" customHeight="1">

</xml_diff>